<commit_message>
fix: workbook table — correct columns, inline dropdowns, click-to-open detail
Table columns: POAM # | Weakness ID | Title | Severity | Status | POC
- Removed Control, Due Date, Milestone, Actions columns from table view (still in export/detail)
- Severity and Status are now inline dropdowns for quick editing
- POC is inline dropdown
- Clicking POAM # or Title opens the detail modal (no separate action buttons)
- Inline select now shows blank placeholder option when no value is set
- Updated test fixture with Weakness Source Identifier column

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-data/test-poam-workbook.xlsx
+++ b/test-data/test-poam-workbook.xlsx
@@ -478,7 +478,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:R11"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -497,6 +497,7 @@
     <col min="15" max="15" width="20.83203125" customWidth="1"/>
     <col min="16" max="16" width="40.83203125" customWidth="1"/>
     <col min="17" max="17" width="20.83203125" customWidth="1"/>
+    <col min="18" max="18" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" xml:space="preserve">
@@ -504,52 +505,55 @@
         <v>Finding Identifier</v>
       </c>
       <c r="B1" t="str">
+        <v>Weakness Source Identifier</v>
+      </c>
+      <c r="C1" t="str">
         <v>Control Family</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Vulnerability Name</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Finding Description</v>
       </c>
-      <c r="E1" t="str" xml:space="preserve">
+      <c r="F1" t="str" xml:space="preserve">
         <v xml:space="preserve">Affected Host(s)
 (For Technical Findings Only)</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Finding Source</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>POC</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Resources Required</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Initial Scheduled Completion Date</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Milestones with Completion Dates</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Changes to Milestones with Completion Dates</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Updated Scheduled Completion Date</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Actual Completion Date</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>Finding Status</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Risk Level</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>Mitigation</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>Comments</v>
       </c>
     </row>
@@ -558,53 +562,56 @@
         <v>POAM-2024-001</v>
       </c>
       <c r="B2" t="str">
+        <v>CVE-2024-24795</v>
+      </c>
+      <c r="C2" t="str">
         <v>CM</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>Apache HTTP Server 2.4.x Multiple Vulnerabilities</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Apache HTTP Server versions prior to 2.4.59 contain multiple vulnerabilities including path traversal and SSRF.</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>web-prod-01, web-prod-02, web-staging-01</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>2024 Annual Security Assessment</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>David Washington</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>Personnel</v>
       </c>
-      <c r="I2" s="1">
+      <c r="J2" s="1">
         <v>45823</v>
       </c>
-      <c r="J2" t="str" xml:space="preserve">
+      <c r="K2" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Patch testing (05/01/2025)
 2. Staging deployment (05/15/2025)
 3. Production rollout (06/15/2025)</v>
       </c>
-      <c r="K2" t="str">
-        <v>N/A</v>
-      </c>
       <c r="L2" t="str">
         <v>N/A</v>
       </c>
       <c r="M2" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
         <v>Ongoing</v>
       </c>
-      <c r="O2" t="str">
+      <c r="P2" t="str">
         <v>Critical</v>
       </c>
-      <c r="P2" t="str">
+      <c r="Q2" t="str">
         <v>Upgrade Apache HTTP Server to version 2.4.59 or later. Apply vendor patches per patch management SOP.</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="R2" t="str">
         <v>Patch approved by CAB. Waiting on maintenance window.</v>
       </c>
     </row>
@@ -613,54 +620,57 @@
         <v>POAM-2024-002</v>
       </c>
       <c r="B3" t="str">
+        <v>QID-38830</v>
+      </c>
+      <c r="C3" t="str">
         <v>AC</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>Weak Password Policy on Domain Controllers</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>Domain password policy does not enforce minimum 14-character passwords or MFA for privileged accounts.</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>N/A</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>2024 DHS ATO Assessment</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>Maria Rodriguez</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>Personnel, Funding</v>
       </c>
-      <c r="I3" s="1">
+      <c r="J3" s="1">
         <v>45777</v>
       </c>
-      <c r="J3" t="str" xml:space="preserve">
+      <c r="K3" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Policy update draft (03/01/2025)
 2. AD GPO changes (03/15/2025)
 3. User notification (04/01/2025)
 4. Enforcement (04/30/2025)</v>
       </c>
-      <c r="K3" t="str">
-        <v/>
-      </c>
-      <c r="L3" s="1">
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" s="1">
         <v>45868</v>
       </c>
-      <c r="M3" t="str">
-        <v/>
-      </c>
       <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
         <v>Ongoing</v>
       </c>
-      <c r="O3" t="str">
+      <c r="P3" t="str">
         <v>High</v>
       </c>
-      <c r="P3" t="str">
+      <c r="Q3" t="str">
         <v>Update AD Group Policy to enforce 14-char minimum. Implement MFA via Azure AD for all privileged accounts.</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="R3" t="str">
         <v>Extended from original date due to MFA vendor procurement delays.</v>
       </c>
     </row>
@@ -669,53 +679,56 @@
         <v>POAM-2024-003</v>
       </c>
       <c r="B4" t="str">
+        <v>NIST-AU-11</v>
+      </c>
+      <c r="C4" t="str">
         <v>AU</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>Insufficient Audit Log Retention</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>System audit logs are retained for only 30 days. NIST 800-53 AU-11 requires minimum 1 year retention.</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>N/A</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>Continuous Monitoring</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>Tom Chen</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>Funding</v>
       </c>
-      <c r="I4" s="1">
+      <c r="J4" s="1">
         <v>45930</v>
       </c>
-      <c r="J4" t="str" xml:space="preserve">
+      <c r="K4" t="str" xml:space="preserve">
         <v xml:space="preserve">1. SIEM storage expansion (07/2025)
 2. Retention policy update (08/2025)
 3. Validation (09/2025)</v>
       </c>
-      <c r="K4" t="str">
+      <c r="L4" t="str">
         <v>N/A</v>
       </c>
-      <c r="L4" t="str">
-        <v/>
-      </c>
       <c r="M4" t="str">
         <v/>
       </c>
       <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
         <v>Ongoing</v>
       </c>
-      <c r="O4" t="str">
+      <c r="P4" t="str">
         <v>Moderate</v>
       </c>
-      <c r="P4" t="str">
+      <c r="Q4" t="str">
         <v>Expand SIEM storage to support 13-month log retention. Update log rotation policy.</v>
       </c>
-      <c r="Q4" t="str">
+      <c r="R4" t="str">
         <v/>
       </c>
     </row>
@@ -724,37 +737,37 @@
         <v>POAM-2024-004</v>
       </c>
       <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
         <v>PE</v>
       </c>
-      <c r="C5" t="str">
+      <c r="D5" t="str">
         <v>Badge Reader Firmware Out of Date</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>Physical access badge readers in Building C are running firmware v2.1, current version is v3.4.</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
         <v>Bldg-C badge readers (12 units)</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>Self-Assessment</v>
       </c>
-      <c r="G5" t="str">
+      <c r="H5" t="str">
         <v>Sarah Patel</v>
       </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
         <v>Funding</v>
       </c>
-      <c r="I5" s="1">
+      <c r="J5" s="1">
         <v>46022</v>
       </c>
-      <c r="J5" t="str" xml:space="preserve">
+      <c r="K5" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Procure firmware licenses (10/2025)
 2. Schedule after-hours update (11/2025)
 3. Test and validate (12/2025)</v>
       </c>
-      <c r="K5" t="str">
-        <v/>
-      </c>
       <c r="L5" t="str">
         <v/>
       </c>
@@ -762,15 +775,18 @@
         <v/>
       </c>
       <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
         <v>Ongoing</v>
       </c>
-      <c r="O5" t="str">
+      <c r="P5" t="str">
         <v>Low</v>
       </c>
-      <c r="P5" t="str">
+      <c r="Q5" t="str">
         <v>Upgrade badge reader firmware to v3.4 per vendor advisory.</v>
       </c>
-      <c r="Q5" t="str">
+      <c r="R5" t="str">
         <v>Low risk — compensating control: security camera coverage.</v>
       </c>
     </row>
@@ -779,53 +795,56 @@
         <v>POAM-2024-005</v>
       </c>
       <c r="B6" t="str">
+        <v>CVE-2022-3602</v>
+      </c>
+      <c r="C6" t="str">
         <v>SI</v>
       </c>
-      <c r="C6" t="str">
+      <c r="D6" t="str">
         <v>OpenSSL 3.0.x Heap Buffer Overflow (CVE-2022-3602)</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>OpenSSL versions 3.0.0-3.0.6 are vulnerable to heap buffer overflow during X.509 certificate verification.</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <v>app-server-01, app-server-02</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>2024 Pen Test</v>
       </c>
-      <c r="G6" t="str">
+      <c r="H6" t="str">
         <v>David Washington</v>
       </c>
-      <c r="H6" t="str">
+      <c r="I6" t="str">
         <v>Personnel</v>
       </c>
-      <c r="I6" s="1">
+      <c r="J6" s="1">
         <v>45657</v>
       </c>
-      <c r="J6" t="str" xml:space="preserve">
+      <c r="K6" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Identify affected systems (10/2024)
 2. Test patches (11/2024)
 3. Deploy (12/2024)</v>
       </c>
-      <c r="K6" t="str">
+      <c r="L6" t="str">
         <v>N/A</v>
       </c>
-      <c r="L6" t="str">
-        <v/>
-      </c>
-      <c r="M6" s="1">
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" s="1">
         <v>45641</v>
       </c>
-      <c r="N6" t="str">
+      <c r="O6" t="str">
         <v>Completed</v>
       </c>
-      <c r="O6" t="str">
+      <c r="P6" t="str">
         <v>Critical</v>
       </c>
-      <c r="P6" t="str">
+      <c r="Q6" t="str">
         <v>Upgraded OpenSSL to 3.0.8 on all affected systems.</v>
       </c>
-      <c r="Q6" t="str">
+      <c r="R6" t="str">
         <v>Verified via Qualys rescan on 12/20/2024. No remaining instances.</v>
       </c>
     </row>
@@ -834,52 +853,55 @@
         <v>POAM-2024-006</v>
       </c>
       <c r="B7" t="str">
+        <v>QID-43012</v>
+      </c>
+      <c r="C7" t="str">
         <v>IA</v>
       </c>
-      <c r="C7" t="str">
+      <c r="D7" t="str">
         <v>Default Credentials on Network Switches</v>
       </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <v>Three network switches found with factory default SNMP community strings.</v>
       </c>
-      <c r="E7" t="str">
+      <c r="F7" t="str">
         <v>sw-floor2-01, sw-floor3-01, sw-floor3-02</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>HVA Assessment</v>
       </c>
-      <c r="G7" t="str">
+      <c r="H7" t="str">
         <v>Tom Chen</v>
       </c>
-      <c r="H7" t="str">
+      <c r="I7" t="str">
         <v>Personnel</v>
       </c>
-      <c r="I7" s="1">
+      <c r="J7" s="1">
         <v>45596</v>
       </c>
-      <c r="J7" t="str" xml:space="preserve">
+      <c r="K7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Inventory switches (09/2024)
 2. Change credentials (10/2024)</v>
       </c>
-      <c r="K7" t="str">
-        <v/>
-      </c>
       <c r="L7" t="str">
         <v/>
       </c>
-      <c r="M7" s="1">
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" s="1">
         <v>45593</v>
       </c>
-      <c r="N7" t="str">
+      <c r="O7" t="str">
         <v>Completed</v>
       </c>
-      <c r="O7" t="str">
+      <c r="P7" t="str">
         <v>High</v>
       </c>
-      <c r="P7" t="str">
+      <c r="Q7" t="str">
         <v>Changed all SNMP community strings to unique complex values. Disabled SNMPv1/v2.</v>
       </c>
-      <c r="Q7" t="str">
+      <c r="R7" t="str">
         <v>Completed ahead of schedule.</v>
       </c>
     </row>
@@ -888,52 +910,55 @@
         <v>POAM-2024-007</v>
       </c>
       <c r="B8" t="str">
+        <v>CVE-2011-3389</v>
+      </c>
+      <c r="C8" t="str">
         <v>SC</v>
       </c>
-      <c r="C8" t="str">
+      <c r="D8" t="str">
         <v>TLS 1.0/1.1 Enabled on Legacy Application</v>
       </c>
-      <c r="D8" t="str">
+      <c r="E8" t="str">
         <v>Legacy payroll application requires TLS 1.0 for client compatibility. Vendor EOL is 2026.</v>
       </c>
-      <c r="E8" t="str">
+      <c r="F8" t="str">
         <v>payroll-legacy-01</v>
       </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
         <v>Continuous Monitoring</v>
       </c>
-      <c r="G8" t="str">
+      <c r="H8" t="str">
         <v>Sarah Patel</v>
       </c>
-      <c r="H8" t="str">
+      <c r="I8" t="str">
         <v>Funding</v>
       </c>
-      <c r="I8" s="1">
+      <c r="J8" s="1">
         <v>45838</v>
       </c>
-      <c r="J8" t="str" xml:space="preserve">
+      <c r="K8" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Vendor engagement for upgrade path (Q1 2025)
 2. Migration planning (Q2 2025)</v>
       </c>
-      <c r="K8" t="str">
+      <c r="L8" t="str">
         <v>Original milestone was Q4 2024. Extended pending vendor response.</v>
       </c>
-      <c r="L8" s="1">
+      <c r="M8" s="1">
         <v>46203</v>
       </c>
-      <c r="M8" t="str">
-        <v/>
-      </c>
       <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
         <v>Risk Accepted</v>
       </c>
-      <c r="O8" t="str">
+      <c r="P8" t="str">
         <v>High</v>
       </c>
-      <c r="P8" t="str">
+      <c r="Q8" t="str">
         <v>Compensating controls: network segmentation, IDS monitoring, restricted access to legacy subnet.</v>
       </c>
-      <c r="Q8" t="str">
+      <c r="R8" t="str">
         <v>Risk accepted by AO on 01/15/2025. Review scheduled for 06/2026.</v>
       </c>
     </row>
@@ -942,53 +967,56 @@
         <v>POAM-2024-008</v>
       </c>
       <c r="B9" t="str">
+        <v>QID-91774</v>
+      </c>
+      <c r="C9" t="str">
         <v>CM</v>
       </c>
-      <c r="C9" t="str">
+      <c r="D9" t="str">
         <v>Unsupported Operating System (Windows Server 2012 R2)</v>
       </c>
-      <c r="D9" t="str">
+      <c r="E9" t="str">
         <v>Two servers running Windows Server 2012 R2 which reached end-of-life October 2023.</v>
       </c>
-      <c r="E9" t="str">
+      <c r="F9" t="str">
         <v>legacy-db-01, legacy-db-02</v>
       </c>
-      <c r="F9" t="str">
+      <c r="G9" t="str">
         <v>Audit</v>
       </c>
-      <c r="G9" t="str">
+      <c r="H9" t="str">
         <v>Maria Rodriguez</v>
       </c>
-      <c r="H9" t="str">
+      <c r="I9" t="str">
         <v>Funding</v>
       </c>
-      <c r="I9" s="1">
+      <c r="J9" s="1">
         <v>45747</v>
       </c>
-      <c r="J9" t="str" xml:space="preserve">
+      <c r="K9" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Migration assessment (01/2025)
 2. New server provisioning (02/2025)
 3. Data migration (03/2025)</v>
       </c>
-      <c r="K9" t="str">
+      <c r="L9" t="str">
         <v>Delayed from original 12/2024 date — budget not approved until Q1 2025.</v>
       </c>
-      <c r="L9" s="1">
+      <c r="M9" s="1">
         <v>45930</v>
       </c>
-      <c r="M9" t="str">
-        <v/>
-      </c>
       <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str">
         <v>Risk Accepted</v>
       </c>
-      <c r="O9" t="str">
+      <c r="P9" t="str">
         <v>Critical</v>
       </c>
-      <c r="P9" t="str">
+      <c r="Q9" t="str">
         <v>ESU licenses purchased. Servers isolated to management VLAN with restricted firewall rules.</v>
       </c>
-      <c r="Q9" t="str">
+      <c r="R9" t="str">
         <v>Risk accepted with compensating controls. Migration funded in FY2025 Q3.</v>
       </c>
     </row>
@@ -997,53 +1025,56 @@
         <v>POAM-2024-009</v>
       </c>
       <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
         <v>RA</v>
       </c>
-      <c r="C10" t="str">
+      <c r="D10" t="str">
         <v>Annual Risk Assessment Not Completed</v>
       </c>
-      <c r="D10" t="str">
+      <c r="E10" t="str">
         <v>Organization has not completed the required annual risk assessment per NIST 800-53 RA-3.</v>
       </c>
-      <c r="E10" t="str">
+      <c r="F10" t="str">
         <v>N/A</v>
       </c>
-      <c r="F10" t="str">
+      <c r="G10" t="str">
         <v>2024 DHS ATO Assessment</v>
       </c>
-      <c r="G10" t="str">
+      <c r="H10" t="str">
         <v>James Lee</v>
       </c>
-      <c r="H10" t="str">
+      <c r="I10" t="str">
         <v>Personnel, Funding</v>
       </c>
-      <c r="I10" s="1">
+      <c r="J10" s="1">
         <v>45747</v>
       </c>
-      <c r="J10" t="str" xml:space="preserve">
+      <c r="K10" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Contract assessor (01/2025)
 2. Conduct assessment (02/2025)
 3. Document findings (03/2025)</v>
       </c>
-      <c r="K10" t="str">
+      <c r="L10" t="str">
         <v>Delayed from 12/2024 — procurement delays for assessment contractor.</v>
       </c>
-      <c r="L10" s="1">
+      <c r="M10" s="1">
         <v>45838</v>
       </c>
-      <c r="M10" t="str">
-        <v/>
-      </c>
       <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
         <v>Delayed</v>
       </c>
-      <c r="O10" t="str">
+      <c r="P10" t="str">
         <v>High</v>
       </c>
-      <c r="P10" t="str">
+      <c r="Q10" t="str">
         <v>Engage third-party assessor to conduct comprehensive risk assessment aligned to NIST SP 800-30.</v>
       </c>
-      <c r="Q10" t="str">
+      <c r="R10" t="str">
         <v>Procurement in progress. Expected contract award 04/2025.</v>
       </c>
     </row>
@@ -1052,38 +1083,38 @@
         <v>POAM-2024-010</v>
       </c>
       <c r="B11" t="str">
+        <v>NIST-SI-3</v>
+      </c>
+      <c r="C11" t="str">
         <v>SI</v>
       </c>
-      <c r="C11" t="str">
+      <c r="D11" t="str">
         <v>Missing Endpoint Detection and Response (EDR)</v>
       </c>
-      <c r="D11" t="str">
+      <c r="E11" t="str">
         <v>Production servers lack EDR/XDR agent deployment. 15 of 42 servers have no endpoint protection.</v>
       </c>
-      <c r="E11" t="str">
+      <c r="F11" t="str">
         <v>Multiple — see asset list</v>
       </c>
-      <c r="F11" t="str">
+      <c r="G11" t="str">
         <v>Continuous Monitoring</v>
       </c>
-      <c r="G11" t="str">
+      <c r="H11" t="str">
         <v>David Washington</v>
       </c>
-      <c r="H11" t="str">
+      <c r="I11" t="str">
         <v>Funding</v>
       </c>
-      <c r="I11" s="1">
+      <c r="J11" s="1">
         <v>45869</v>
       </c>
-      <c r="J11" t="str" xml:space="preserve">
+      <c r="K11" t="str" xml:space="preserve">
         <v xml:space="preserve">1. EDR license procurement (04/2025)
 2. Pilot deployment (05/2025)
 3. Full rollout (06/2025)
 4. Validation (07/2025)</v>
       </c>
-      <c r="K11" t="str">
-        <v/>
-      </c>
       <c r="L11" t="str">
         <v/>
       </c>
@@ -1091,21 +1122,24 @@
         <v/>
       </c>
       <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
         <v>Ongoing</v>
       </c>
-      <c r="O11" t="str">
+      <c r="P11" t="str">
         <v>Critical</v>
       </c>
-      <c r="P11" t="str">
+      <c r="Q11" t="str">
         <v>Deploy CrowdStrike Falcon agent to all production servers. Update baseline configuration.</v>
       </c>
-      <c r="Q11" t="str">
+      <c r="R11" t="str">
         <v>Budget approved. Licenses ordered.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>